<commit_message>
Finance update 2026-06-12 12:19
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -15,7 +15,6 @@
     <sheet name="Loans" sheetId="10" r:id="rId10"/>
     <sheet name="LoanPayments" sheetId="11" r:id="rId11"/>
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
-    <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -524,57 +523,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-      <c r="F1" t="str">
-        <v>notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>mqarvl0ed5l</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2025-01-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Zaggle Amount</v>
-      </c>
-      <c r="D2">
-        <v>100000</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P2"/>
@@ -791,6 +739,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
@@ -830,16 +788,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mqamhld44k0</v>
+        <v>mqamidmqnc1</v>
       </c>
       <c r="B2" t="str">
         <v>2024-01-01</v>
       </c>
       <c r="C2" t="str">
-        <v>Kite</v>
+        <v>Coin</v>
       </c>
       <c r="D2">
-        <v>724093</v>
+        <v>102495</v>
       </c>
       <c r="E2" t="str">
         <v>Active</v>
@@ -870,7 +828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K2"/>
   <sheetData>
@@ -911,87 +869,6 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mqamidmqnc1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2024-01-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Coin</v>
-      </c>
-      <c r="D2">
-        <v>102495</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-      <c r="F1" t="str">
-        <v>details</v>
-      </c>
-      <c r="G1" t="str">
-        <v>returnDate</v>
-      </c>
-      <c r="H1" t="str">
-        <v>returnAmount</v>
-      </c>
-      <c r="I1" t="str">
-        <v>returnInterest</v>
-      </c>
-      <c r="J1" t="str">
-        <v>reinvestedInto</v>
-      </c>
-      <c r="K1" t="str">
-        <v>reinvestNote</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
         <v>mqary2elefu</v>
       </c>
       <c r="B2" t="str">

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:20
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -696,57 +696,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>month</v>
-      </c>
-      <c r="D1" t="str">
-        <v>type</v>
-      </c>
-      <c r="E1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="F1" t="str">
-        <v>source</v>
-      </c>
-      <c r="G1" t="str">
-        <v>notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>mqaswa6dn63</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2026-01-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2026-01</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="E2">
-        <v>217000</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finance update 2026-06-12 12:24
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -408,10 +408,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>bank</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>source</v>
+      </c>
+      <c r="G1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqawesn9wbg</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>SBI</v>
+      </c>
+      <c r="D2">
+        <v>392398</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:25
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -525,7 +525,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -567,9 +567,29 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>mqawgcf8tnd</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Angle</v>
+      </c>
+      <c r="D3">
+        <v>28320</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:26
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -606,10 +606,51 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  <dimension ref="A1:F2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqawh8gkg3b</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>LIC</v>
+      </c>
+      <c r="D2">
+        <v>891265</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:28
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Loans" sheetId="10" r:id="rId10"/>
     <sheet name="LoanPayments" sheetId="11" r:id="rId11"/>
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
+    <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -493,6 +494,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:30
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,10 +547,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  <dimension ref="A1:I2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>fdNumber</v>
+      </c>
+      <c r="D1" t="str">
+        <v>bank</v>
+      </c>
+      <c r="E1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="F1" t="str">
+        <v>rate</v>
+      </c>
+      <c r="G1" t="str">
+        <v>status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>source</v>
+      </c>
+      <c r="I1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqawn51h6j5</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-08-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>HDFC - 48487</v>
+      </c>
+      <c r="D2" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E2">
+        <v>83363</v>
+      </c>
+      <c r="F2">
+        <v>6.25</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:31
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -607,9 +607,38 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>mqawohloy5s</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2025-07-05</v>
+      </c>
+      <c r="C3" t="str">
+        <v>HDFC - 41503</v>
+      </c>
+      <c r="D3" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E3">
+        <v>23807</v>
+      </c>
+      <c r="F3">
+        <v>6.25</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:32
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -636,9 +636,38 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqawpo3ld8x</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2025-06-25</v>
+      </c>
+      <c r="C4" t="str">
+        <v>HDFC - 360479</v>
+      </c>
+      <c r="D4" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E4">
+        <v>59515</v>
+      </c>
+      <c r="F4">
+        <v>6.25</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:35
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -665,9 +665,38 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mqawspdh4el</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2025-06-25</v>
+      </c>
+      <c r="C5" t="str">
+        <v>HDFC - 59185</v>
+      </c>
+      <c r="D5" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E5">
+        <v>59523</v>
+      </c>
+      <c r="F5">
+        <v>6.25</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:36
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -723,9 +723,38 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mqawukv8i1i</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2025-07-31</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HDFC - 1710</v>
+      </c>
+      <c r="D7" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E7">
+        <v>15920</v>
+      </c>
+      <c r="F7">
+        <v>6.26</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:37
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -752,9 +752,38 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>mqawvkcv1q1</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2025-07-31</v>
+      </c>
+      <c r="C8" t="str">
+        <v>HDFC - 71532</v>
+      </c>
+      <c r="D8" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E8">
+        <v>16446</v>
+      </c>
+      <c r="F8">
+        <v>6.26</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:40
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -781,9 +781,38 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>mqawztfpujf</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2025-08-29</v>
+      </c>
+      <c r="C9" t="str">
+        <v>HDFC - 0925</v>
+      </c>
+      <c r="D9" t="str">
+        <v>HDFC</v>
+      </c>
+      <c r="E9">
+        <v>55000</v>
+      </c>
+      <c r="F9">
+        <v>6.25</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:47
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -810,9 +810,38 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>mqax8bx1l3o</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2025-08-11</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Axis</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Axis</v>
+      </c>
+      <c r="E10">
+        <v>114481</v>
+      </c>
+      <c r="F10">
+        <v>6.25</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:48
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -839,9 +839,38 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>mqax9iloxsz</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2025-01-11</v>
+      </c>
+      <c r="C11" t="str">
+        <v>PNB - 0626</v>
+      </c>
+      <c r="D11" t="str">
+        <v>PNB</v>
+      </c>
+      <c r="E11">
+        <v>51358</v>
+      </c>
+      <c r="F11">
+        <v>6.8</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 12:49
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -897,9 +897,38 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>mqaxbd0900v</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2025-01-10</v>
+      </c>
+      <c r="C13" t="str">
+        <v>PNB - 1207</v>
+      </c>
+      <c r="D13" t="str">
+        <v>PNB</v>
+      </c>
+      <c r="E13">
+        <v>10000</v>
+      </c>
+      <c r="F13">
+        <v>6.8</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:04
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,10 +935,63 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>rate</v>
+      </c>
+      <c r="F1" t="str">
+        <v>status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>source</v>
+      </c>
+      <c r="H1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqaxu3z8clp</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2024-08-20</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D2">
+        <v>100000</v>
+      </c>
+      <c r="E2">
+        <v>18</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:05
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1015,9 +1015,35 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqaxvk3o0vz</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2024-09-08</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D4">
+        <v>125000</v>
+      </c>
+      <c r="E4">
+        <v>18</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:06
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1067,9 +1067,35 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>mqaxwvqolcl</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2024-09-23</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D6">
+        <v>100000</v>
+      </c>
+      <c r="E6">
+        <v>18</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:07
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1093,9 +1093,35 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mqaxydf8n0m</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2024-10-03</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D7">
+        <v>100000</v>
+      </c>
+      <c r="E7">
+        <v>18</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:08
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1145,9 +1145,35 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>mqaxzg24ekz</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2024-10-13</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D9">
+        <v>100000</v>
+      </c>
+      <c r="E9">
+        <v>18</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:09
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1197,9 +1197,35 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>mqay0w444pi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2024-11-13</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D11">
+        <v>80000</v>
+      </c>
+      <c r="E11">
+        <v>18</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:10
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1249,9 +1249,35 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>mqay1x6kq2v</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2025-12-02</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D13">
+        <v>100000</v>
+      </c>
+      <c r="E13">
+        <v>18</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:11
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1301,9 +1301,35 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>mqay3578igw</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2024-12-13</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D15">
+        <v>100000</v>
+      </c>
+      <c r="E15">
+        <v>18</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:14
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1327,9 +1327,35 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>mqay6x5wr46</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2025-03-29</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D16">
+        <v>200000</v>
+      </c>
+      <c r="E16">
+        <v>18</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:15
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1379,9 +1379,35 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>mqay852svv3</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2025-04-16</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D18">
+        <v>53000</v>
+      </c>
+      <c r="E18">
+        <v>18</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:16
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:L2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,6 +433,21 @@
       <c r="G1" t="str">
         <v>details</v>
       </c>
+      <c r="H1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="I1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="J1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="K1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="L1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,10 +471,25 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -547,7 +577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:P13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,9 +602,30 @@
         <v>status</v>
       </c>
       <c r="H1" t="str">
+        <v>brokenDate</v>
+      </c>
+      <c r="I1" t="str">
+        <v>brokenAmount</v>
+      </c>
+      <c r="J1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="K1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="L1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="M1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="N1" t="str">
+        <v>reinvestNote</v>
+      </c>
+      <c r="O1" t="str">
         <v>source</v>
       </c>
-      <c r="I1" t="str">
+      <c r="P1" t="str">
         <v>details</v>
       </c>
     </row>
@@ -603,7 +654,28 @@
       <c r="H2" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v/>
       </c>
     </row>
@@ -632,7 +704,28 @@
       <c r="H3" t="str">
         <v/>
       </c>
-      <c r="I3" t="str">
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v/>
       </c>
     </row>
@@ -661,7 +754,28 @@
       <c r="H4" t="str">
         <v/>
       </c>
-      <c r="I4" t="str">
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v/>
       </c>
     </row>
@@ -690,7 +804,28 @@
       <c r="H5" t="str">
         <v/>
       </c>
-      <c r="I5" t="str">
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v/>
       </c>
     </row>
@@ -719,7 +854,28 @@
       <c r="H6" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
         <v/>
       </c>
     </row>
@@ -748,7 +904,28 @@
       <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I7" t="str">
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
         <v/>
       </c>
     </row>
@@ -777,7 +954,28 @@
       <c r="H8" t="str">
         <v/>
       </c>
-      <c r="I8" t="str">
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
         <v/>
       </c>
     </row>
@@ -806,7 +1004,28 @@
       <c r="H9" t="str">
         <v/>
       </c>
-      <c r="I9" t="str">
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
         <v/>
       </c>
     </row>
@@ -835,7 +1054,28 @@
       <c r="H10" t="str">
         <v/>
       </c>
-      <c r="I10" t="str">
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
         <v/>
       </c>
     </row>
@@ -864,7 +1104,28 @@
       <c r="H11" t="str">
         <v/>
       </c>
-      <c r="I11" t="str">
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
         <v/>
       </c>
     </row>
@@ -893,7 +1154,28 @@
       <c r="H12" t="str">
         <v/>
       </c>
-      <c r="I12" t="str">
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
         <v/>
       </c>
     </row>
@@ -922,20 +1204,41 @@
       <c r="H13" t="str">
         <v/>
       </c>
-      <c r="I13" t="str">
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:M18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -962,6 +1265,21 @@
       <c r="H1" t="str">
         <v>details</v>
       </c>
+      <c r="I1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="J1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="K1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="L1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="M1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -988,6 +1306,21 @@
       <c r="H2" t="str">
         <v/>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1014,6 +1347,21 @@
       <c r="H3" t="str">
         <v/>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1040,6 +1388,21 @@
       <c r="H4" t="str">
         <v/>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1066,6 +1429,21 @@
       <c r="H5" t="str">
         <v/>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1092,6 +1470,21 @@
       <c r="H6" t="str">
         <v/>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1118,6 +1511,21 @@
       <c r="H7" t="str">
         <v/>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1144,6 +1552,21 @@
       <c r="H8" t="str">
         <v/>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1170,6 +1593,21 @@
       <c r="H9" t="str">
         <v/>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1196,6 +1634,21 @@
       <c r="H10" t="str">
         <v/>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1222,6 +1675,21 @@
       <c r="H11" t="str">
         <v/>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1248,6 +1716,21 @@
       <c r="H12" t="str">
         <v/>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1274,6 +1757,21 @@
       <c r="H13" t="str">
         <v/>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1300,6 +1798,21 @@
       <c r="H14" t="str">
         <v/>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1326,6 +1839,21 @@
       <c r="H15" t="str">
         <v/>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1352,6 +1880,21 @@
       <c r="H16" t="str">
         <v/>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1378,13 +1921,28 @@
       <c r="H17" t="str">
         <v/>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
         <v>mqay852svv3</v>
       </c>
       <c r="B18" t="str">
-        <v>2025-04-16</v>
+        <v>2025-04-26</v>
       </c>
       <c r="C18" t="str">
         <v>Gold Fin</v>
@@ -1404,10 +1962,25 @@
       <c r="H18" t="str">
         <v/>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1424,7 +1997,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:K3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1445,6 +2018,21 @@
       <c r="F1" t="str">
         <v>details</v>
       </c>
+      <c r="G1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="I1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="J1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="K1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1465,6 +2053,21 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1485,17 +2088,32 @@
       <c r="F3" t="str">
         <v/>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1516,6 +2134,21 @@
       <c r="F1" t="str">
         <v>details</v>
       </c>
+      <c r="G1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="I1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="J1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="K1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1536,17 +2169,32 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1567,6 +2215,21 @@
       <c r="F1" t="str">
         <v>details</v>
       </c>
+      <c r="G1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="I1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="J1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="K1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1587,10 +2250,25 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:17
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2004,9 +2004,35 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>mqayayadcct</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2025-05-08</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D20">
+        <v>90000</v>
+      </c>
+      <c r="E20">
+        <v>18</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:18
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2082,9 +2082,35 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>mqaycnfw52m</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2025-05-24</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D23">
+        <v>200000</v>
+      </c>
+      <c r="E23">
+        <v>18</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:19
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2108,9 +2108,35 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>mqaydc7w8hu</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2025-06-02</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D24">
+        <v>100000</v>
+      </c>
+      <c r="E24">
+        <v>18</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:20
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2186,9 +2186,35 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>mqayevqd5cv</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2025-07-07</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D27">
+        <v>100000</v>
+      </c>
+      <c r="E27">
+        <v>18</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:21
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2212,9 +2212,35 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>mqayh1akrkz</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D28">
+        <v>100000</v>
+      </c>
+      <c r="E28">
+        <v>18</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:22
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2238,9 +2238,35 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>mqayhuwcyrq</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2025-05-02</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D29">
+        <v>130000</v>
+      </c>
+      <c r="E29">
+        <v>18</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-12 13:26
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2264,9 +2264,35 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>mqaymnt9tf7</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2024-12-02</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D30">
+        <v>100000</v>
+      </c>
+      <c r="E30">
+        <v>18</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 04:58
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2003,6 +2003,21 @@
       <c r="H19" t="str">
         <v/>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2029,6 +2044,21 @@
       <c r="H20" t="str">
         <v/>
       </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2055,6 +2085,21 @@
       <c r="H21" t="str">
         <v/>
       </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2081,6 +2126,21 @@
       <c r="H22" t="str">
         <v/>
       </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2107,6 +2167,21 @@
       <c r="H23" t="str">
         <v/>
       </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2133,6 +2208,21 @@
       <c r="H24" t="str">
         <v/>
       </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2159,6 +2249,21 @@
       <c r="H25" t="str">
         <v/>
       </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2185,6 +2290,21 @@
       <c r="H26" t="str">
         <v/>
       </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2211,6 +2331,21 @@
       <c r="H27" t="str">
         <v/>
       </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2237,6 +2372,21 @@
       <c r="H28" t="str">
         <v/>
       </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2263,6 +2413,21 @@
       <c r="H29" t="str">
         <v/>
       </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2287,6 +2452,21 @@
         <v/>
       </c>
       <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
         <v/>
       </c>
     </row>
@@ -2299,10 +2479,63 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>person</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>rate</v>
+      </c>
+      <c r="F1" t="str">
+        <v>status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>source</v>
+      </c>
+      <c r="H1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbvxx40xin</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2023-05-09</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Shiva Sumanth</v>
+      </c>
+      <c r="D2">
+        <v>200000</v>
+      </c>
+      <c r="E2">
+        <v>24</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:00
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2470,9 +2470,35 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>mqbw09mw8r8</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Gold Fin</v>
+      </c>
+      <c r="D31">
+        <v>65000</v>
+      </c>
+      <c r="E31">
+        <v>18</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:04
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2559,9 +2559,35 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>mqbw5a601ln</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2025-08-05</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Venky Gudur</v>
+      </c>
+      <c r="D3">
+        <v>150000</v>
+      </c>
+      <c r="E3">
+        <v>18</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:06
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2585,9 +2585,35 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqbw7xe8sgy</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Prasanth USA</v>
+      </c>
+      <c r="D4">
+        <v>150000</v>
+      </c>
+      <c r="E4">
+        <v>25</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:07
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2611,9 +2611,35 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mqbw8t5j9rm</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2025-04-22</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Prasanth USA</v>
+      </c>
+      <c r="D5">
+        <v>70000</v>
+      </c>
+      <c r="E5">
+        <v>24</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:08
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2637,9 +2637,35 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>mqbw9uq7j2v</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2025-04-04</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sravani</v>
+      </c>
+      <c r="D6">
+        <v>25000</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:10
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2663,9 +2663,35 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mqbwcbj3wnr</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2025-12-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Shiva Sumanth</v>
+      </c>
+      <c r="D7">
+        <v>400000</v>
+      </c>
+      <c r="E7">
+        <v>18</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:14
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2689,9 +2689,35 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>mqbwibfr9lp</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-05-27</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Sumanth</v>
+      </c>
+      <c r="D8">
+        <v>600000</v>
+      </c>
+      <c r="E8">
+        <v>18</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:16
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2715,9 +2715,35 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>mqbwkbw8fnc</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Suresh Anna</v>
+      </c>
+      <c r="D9">
+        <v>600000</v>
+      </c>
+      <c r="E9">
+        <v>18</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:19
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2741,9 +2741,35 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>mqbwp3fzt4s</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2025-08-30</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Nag Vitech</v>
+      </c>
+      <c r="D10">
+        <v>300000</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:21
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2505,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2767,9 +2767,35 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>mqbwr9e0eq3</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Vamsi Kurapti</v>
+      </c>
+      <c r="D11">
+        <v>400000</v>
+      </c>
+      <c r="E11">
+        <v>24</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:24
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -16,6 +16,7 @@
     <sheet name="LoanPayments" sheetId="11" r:id="rId11"/>
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
     <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
+    <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -575,6 +576,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P13"/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:25
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -578,10 +578,57 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="G1" t="str">
+        <v>returns</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbwvwohab1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-11-22</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Golden Homes</v>
+      </c>
+      <c r="D2">
+        <v>3200000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:38
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -578,57 +578,10 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-      <c r="F1" t="str">
-        <v>notes</v>
-      </c>
-      <c r="G1" t="str">
-        <v>returns</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>mqbwvwohab1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2025-11-22</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Golden Homes</v>
-      </c>
-      <c r="D2">
-        <v>3200000</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2553,6 +2506,21 @@
       <c r="H31" t="str">
         <v/>
       </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -2563,7 +2531,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:M11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2590,6 +2558,21 @@
       <c r="H1" t="str">
         <v>details</v>
       </c>
+      <c r="I1" t="str">
+        <v>returnDate</v>
+      </c>
+      <c r="J1" t="str">
+        <v>returnAmount</v>
+      </c>
+      <c r="K1" t="str">
+        <v>returnInterest</v>
+      </c>
+      <c r="L1" t="str">
+        <v>reinvestedInto</v>
+      </c>
+      <c r="M1" t="str">
+        <v>reinvestNote</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2616,6 +2599,21 @@
       <c r="H2" t="str">
         <v/>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2642,6 +2640,21 @@
       <c r="H3" t="str">
         <v/>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2668,6 +2681,21 @@
       <c r="H4" t="str">
         <v/>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2694,6 +2722,21 @@
       <c r="H5" t="str">
         <v/>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2720,6 +2763,21 @@
       <c r="H6" t="str">
         <v/>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2746,6 +2804,21 @@
       <c r="H7" t="str">
         <v/>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2772,6 +2845,21 @@
       <c r="H8" t="str">
         <v/>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2798,6 +2886,21 @@
       <c r="H9" t="str">
         <v/>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2824,6 +2927,21 @@
       <c r="H10" t="str">
         <v/>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2850,10 +2968,25 @@
       <c r="H11" t="str">
         <v/>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:39
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -16,6 +16,7 @@
     <sheet name="LoanPayments" sheetId="11" r:id="rId11"/>
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
     <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
+    <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -575,6 +576,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P13"/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:40
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -578,10 +578,57 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="G1" t="str">
+        <v>returns_rate</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbxfp9z8n9</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-11-22</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Golden Home Projects</v>
+      </c>
+      <c r="D2">
+        <v>3200000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:44
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
     <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
     <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
+    <sheet name="PF_Amount" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -633,6 +634,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P13"/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:49
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -636,10 +636,57 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="G1" t="str">
+        <v>returns</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbxqggnpkv</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-12-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>PF Till 2025</v>
+      </c>
+      <c r="D2">
+        <v>380000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 05:58
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3386,10 +3386,57 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>month</v>
+      </c>
+      <c r="D1" t="str">
+        <v>type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="F1" t="str">
+        <v>source</v>
+      </c>
+      <c r="G1" t="str">
+        <v>notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqby2c9k2f1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-01-30</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-01</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E2">
+        <v>217000</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finance update 2026-06-13 05:59
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3386,7 +3386,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3457,9 +3457,32 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqby47coun3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-03</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E4">
+        <v>355278</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>F&amp;F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finance update 2026-06-13 06:00
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3386,7 +3386,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3480,9 +3480,32 @@
         <v>F&amp;F</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mqby59pj5vj</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-06</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E5">
+        <v>2157464</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>F&amp;F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finance update 2026-06-13 06:04
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3386,7 +3386,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3526,9 +3526,32 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mqby9xc0g9a</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-31</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-06</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Interest Received</v>
+      </c>
+      <c r="E7">
+        <v>194980</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>Interest Amounts Till 13/06/2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finance update 2026-06-13 06:05
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3376,10 +3376,51 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:F2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>category</v>
+      </c>
+      <c r="E1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbybp5jv4p</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Expense till Date</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="E2">
+        <v>107900</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 06:07
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2636,7 +2636,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3089,9 +3089,35 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>mqbyea4ngqv</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-01-29</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Balu CSE</v>
+      </c>
+      <c r="D12">
+        <v>10000</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 06:08
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2636,7 +2636,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3115,9 +3115,35 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>mqbyf34ouje</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-01-11</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Masthan</v>
+      </c>
+      <c r="D13">
+        <v>5000</v>
+      </c>
+      <c r="E13">
+        <v>24</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 06:19
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
     <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
     <sheet name="PF_Amount" sheetId="15" r:id="rId15"/>
+    <sheet name="GoldLoanRe_Payments" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -691,6 +692,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P13"/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 06:22
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -694,10 +694,45 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbyx1wo9xl</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Gold Loan Repayment Till Date</v>
+      </c>
+      <c r="D2">
+        <v>699344</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:49
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1391,9 +1391,38 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>mqcalqnmldy</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2025-08-14</v>
+      </c>
+      <c r="C14" t="str">
+        <v>305002118270(92453)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E14">
+        <v>30000</v>
+      </c>
+      <c r="F14">
+        <v>7.65</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3160,6 +3189,21 @@
       <c r="H12" t="str">
         <v/>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -3184,6 +3228,21 @@
         <v/>
       </c>
       <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:50
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1413,16 +1413,66 @@
       <c r="G14" t="str">
         <v>Active</v>
       </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
       <c r="O14" t="str">
         <v/>
       </c>
       <c r="P14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>mqcanwk2tpa</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2025-08-14</v>
+      </c>
+      <c r="C15" t="str">
+        <v>305002118269(92452)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E15">
+        <v>50000</v>
+      </c>
+      <c r="F15">
+        <v>7.65</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:52
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1470,9 +1470,38 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>mqcap9qaibn</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2025-08-14</v>
+      </c>
+      <c r="C16" t="str">
+        <v>305002118247(92451)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E16">
+        <v>50000</v>
+      </c>
+      <c r="F16">
+        <v>7.65</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:53
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1499,9 +1499,38 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>mqcar3qqnhm</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2025-08-14</v>
+      </c>
+      <c r="C17" t="str">
+        <v>305002118236(92450)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E17">
+        <v>50000</v>
+      </c>
+      <c r="F17">
+        <v>7.65</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:54
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1528,9 +1528,38 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>mqcasw4p322</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2025-08-14</v>
+      </c>
+      <c r="C18" t="str">
+        <v>305002118225(92449)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E18">
+        <v>50000</v>
+      </c>
+      <c r="F18">
+        <v>7.65</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:56
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1557,9 +1557,38 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>mqcauelml86</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2025-08-20</v>
+      </c>
+      <c r="C19" t="str">
+        <v>305002125833(92459)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E19">
+        <v>50000</v>
+      </c>
+      <c r="F19">
+        <v>7.65</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:57
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1586,9 +1586,38 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>mqcavvbv0ms</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2025-08-20</v>
+      </c>
+      <c r="C20" t="str">
+        <v>305002125822(92460)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E20">
+        <v>50000</v>
+      </c>
+      <c r="F20">
+        <v>7.65</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:58
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1615,9 +1615,38 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>mqcaxjsyw5w</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2025-08-20</v>
+      </c>
+      <c r="C21" t="str">
+        <v>305002125811(92461)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E21">
+        <v>50000</v>
+      </c>
+      <c r="F21">
+        <v>7.65</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 11:59
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1644,9 +1644,38 @@
         <v/>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>mqcayxtejwi</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2025-08-20</v>
+      </c>
+      <c r="C22" t="str">
+        <v>305002125800(92462)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E22">
+        <v>50000</v>
+      </c>
+      <c r="F22">
+        <v>7.65</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:00
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1673,9 +1673,38 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>mqcb09hep49</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2025-08-20</v>
+      </c>
+      <c r="C23" t="str">
+        <v>305002125844(92463)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E23">
+        <v>66500</v>
+      </c>
+      <c r="F23">
+        <v>7.65</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:06
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1702,9 +1702,38 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>mqcb8b4hxsw</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="C24" t="str">
+        <v>305002613285(92503)</v>
+      </c>
+      <c r="D24" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E24">
+        <v>100000</v>
+      </c>
+      <c r="F24">
+        <v>7.65</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:07
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1731,9 +1731,38 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>mqcb9pd6bjv</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C25" t="str">
+        <v>305002593197(92494)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E25">
+        <v>500000</v>
+      </c>
+      <c r="F25">
+        <v>7.65</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:09
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1760,9 +1760,38 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>mqcbb42p4zi</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="C26" t="str">
+        <v>305002594395(92499)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E26">
+        <v>200000</v>
+      </c>
+      <c r="F26">
+        <v>7.65</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:10
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1789,9 +1789,38 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>mqcbcl8yj9m</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2025-04-30</v>
+      </c>
+      <c r="C27" t="str">
+        <v>305002594384(92497)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E27">
+        <v>250000</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:11
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1818,9 +1818,38 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>mqcbefyiplw</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="C28" t="str">
+        <v>305002594373(92496)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E28">
+        <v>150000</v>
+      </c>
+      <c r="F28">
+        <v>7.65</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:12
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1847,9 +1847,38 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>mqcbfvuivx6</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="C29" t="str">
+        <v>305002613434(92506)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>DCC</v>
+      </c>
+      <c r="E29">
+        <v>86298</v>
+      </c>
+      <c r="F29">
+        <v>7.65</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:51
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1794,7 +1794,7 @@
         <v>mqcbcl8yj9m</v>
       </c>
       <c r="B27" t="str">
-        <v>2025-04-30</v>
+        <v>2026-04-30</v>
       </c>
       <c r="C27" t="str">
         <v>305002594384(92497)</v>
@@ -1806,7 +1806,7 @@
         <v>250000</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>7.65</v>
       </c>
       <c r="G27" t="str">
         <v>Active</v>

</xml_diff>

<commit_message>
Finance update 2026-06-13 12:56
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1463,6 +1463,27 @@
       <c r="G15" t="str">
         <v>Active</v>
       </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
       <c r="O15" t="str">
         <v/>
       </c>
@@ -1492,6 +1513,27 @@
       <c r="G16" t="str">
         <v>Active</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
       <c r="O16" t="str">
         <v/>
       </c>
@@ -1521,6 +1563,27 @@
       <c r="G17" t="str">
         <v>Active</v>
       </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
       <c r="O17" t="str">
         <v/>
       </c>
@@ -1550,6 +1613,27 @@
       <c r="G18" t="str">
         <v>Active</v>
       </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
       <c r="O18" t="str">
         <v/>
       </c>
@@ -1579,6 +1663,27 @@
       <c r="G19" t="str">
         <v>Active</v>
       </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
       <c r="O19" t="str">
         <v/>
       </c>
@@ -1608,6 +1713,27 @@
       <c r="G20" t="str">
         <v>Active</v>
       </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
       <c r="O20" t="str">
         <v/>
       </c>
@@ -1637,6 +1763,27 @@
       <c r="G21" t="str">
         <v>Active</v>
       </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
       <c r="O21" t="str">
         <v/>
       </c>
@@ -1666,6 +1813,27 @@
       <c r="G22" t="str">
         <v>Active</v>
       </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
       <c r="O22" t="str">
         <v/>
       </c>
@@ -1695,6 +1863,27 @@
       <c r="G23" t="str">
         <v>Active</v>
       </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
       <c r="O23" t="str">
         <v/>
       </c>
@@ -1724,6 +1913,27 @@
       <c r="G24" t="str">
         <v>Active</v>
       </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
       <c r="O24" t="str">
         <v/>
       </c>
@@ -1753,6 +1963,27 @@
       <c r="G25" t="str">
         <v>Active</v>
       </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
       <c r="O25" t="str">
         <v/>
       </c>
@@ -1782,6 +2013,27 @@
       <c r="G26" t="str">
         <v>Active</v>
       </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
       <c r="O26" t="str">
         <v/>
       </c>
@@ -1794,7 +2046,7 @@
         <v>mqcbcl8yj9m</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-04-30</v>
+        <v>2025-04-30</v>
       </c>
       <c r="C27" t="str">
         <v>305002594384(92497)</v>
@@ -1810,6 +2062,27 @@
       </c>
       <c r="G27" t="str">
         <v>Active</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
       </c>
       <c r="O27" t="str">
         <v/>
@@ -1840,6 +2113,27 @@
       <c r="G28" t="str">
         <v>Active</v>
       </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
       <c r="O28" t="str">
         <v/>
       </c>
@@ -1868,6 +2162,27 @@
       </c>
       <c r="G29" t="str">
         <v>Active</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
       </c>
       <c r="O29" t="str">
         <v/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:03
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -19,6 +19,7 @@
     <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
     <sheet name="PF_Amount" sheetId="15" r:id="rId15"/>
     <sheet name="GoldLoanRe_Payments" sheetId="16" r:id="rId16"/>
+    <sheet name="Partial_Outs" sheetId="17" r:id="rId17"/>
   </sheets>
 </workbook>
 </file>
@@ -737,6 +738,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P29"/>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:04
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -740,10 +740,51 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:F2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqcdablhtac</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C2" t="str">
+        <v xml:space="preserve">Fire NOC - Sumanth </v>
+      </c>
+      <c r="D2">
+        <v>5200</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:05
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -740,7 +740,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -802,9 +802,29 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqcdbzsu86a</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C4" t="str">
+        <v>spiktic tank cleaning</v>
+      </c>
+      <c r="D4">
+        <v>14300</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:16
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -740,7 +740,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -842,9 +842,29 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>mqcdpou6y7h</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Bnglr site visit</v>
+      </c>
+      <c r="D6">
+        <v>8000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:57
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3614,7 +3614,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4149,9 +4149,35 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>mqcf6af1t2r</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Nag Vitech</v>
+      </c>
+      <c r="D14">
+        <v>50000</v>
+      </c>
+      <c r="E14">
+        <v>24</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 13:59
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -740,7 +740,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -862,9 +862,29 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mqcf9sbxro4</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Sumanth Bal for temple</v>
+      </c>
+      <c r="D7">
+        <v>8500</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-13 14:00
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -740,7 +740,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -882,9 +882,29 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>mqcfa6x1ksb</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Sumanth Phonepay</v>
+      </c>
+      <c r="D8">
+        <v>2170</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-15 05:11
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -4214,6 +4214,21 @@
       <c r="H14" t="str">
         <v/>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -4502,7 +4517,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4544,9 +4559,29 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>mqer9ftbadd</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-14</v>
+      </c>
+      <c r="C3" t="str">
+        <v>For Balu Daughter</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3">
+        <v>2500</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-15 05:14
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -4517,7 +4517,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4579,9 +4579,29 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>mqere4jt2e9</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C4" t="str">
+        <v>HarithGas &amp; Travel</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4">
+        <v>5000</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-15 07:04
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -15,11 +15,12 @@
     <sheet name="Loans" sheetId="10" r:id="rId10"/>
     <sheet name="LoanPayments" sheetId="11" r:id="rId11"/>
     <sheet name="CashFlow" sheetId="12" r:id="rId12"/>
-    <sheet name="Zaggle" sheetId="13" r:id="rId13"/>
-    <sheet name="GoldenHome" sheetId="14" r:id="rId14"/>
-    <sheet name="PF_Amount" sheetId="15" r:id="rId15"/>
-    <sheet name="GoldLoanRe_Payments" sheetId="16" r:id="rId16"/>
-    <sheet name="Partial_Outs" sheetId="17" r:id="rId17"/>
+    <sheet name="_CustomDefs" sheetId="13" r:id="rId13"/>
+    <sheet name="Zaggle" sheetId="14" r:id="rId14"/>
+    <sheet name="GoldenHome" sheetId="15" r:id="rId15"/>
+    <sheet name="PF_Amount" sheetId="16" r:id="rId16"/>
+    <sheet name="GoldLoanRe_Payments" sheetId="17" r:id="rId17"/>
+    <sheet name="Partial_Outs" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -530,58 +531,28 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:A2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-      <c r="F1" t="str">
-        <v>notes</v>
+        <v>defsJson</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mqawkf50bya</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2024-01-01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Zaggle</v>
-      </c>
-      <c r="D2">
-        <v>120896</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
+        <v>[{"id":"mqawjyxgccd","name":"Zaggle","icon":"🏆","sectionType":"investment","sheetName":"Zaggle","columns":[{"key":"date","label":"Date","type":"date"},{"key":"name","label":"Name","type":"text"},{"key":"amount","label":"Amount","type":"number"},{"key":"status","label":"Status","type":"status"},{"key":"notes","label":"Notes / Other Details","type":"text"}]},{"id":"mqbxdl2o7x8","name":"GoldenHome","icon":"🏠","sectionType":"investment","sheetName":"GoldenHome","columns":[{"key":"date","label":"Date","type":"date"},{"key":"name","label":"Name","type":"text"},{"key":"amount","label":"Amount","type":"number"},{"key":"status","label":"Status","type":"status"},{"key":"notes","label":"Notes / Other Details","type":"text"},{"key":"returns_rate","label":"Returns Rate","type":"rate"}]},{"id":"mqbxl7zznrv","name":"PF Amount","icon":"💎","sectionType":"investment","sheetName":"PF_Amount","columns":[{"key":"date","label":"Date","type":"date"},{"key":"name","label":"Name","type":"text"},{"key":"amount","label":"Amount","type":"number"},{"key":"status","label":"Status","type":"status"},{"key":"notes","label":"Notes / Other Details","type":"text"},{"key":"returns","label":"Returns","type":"rate"}]},{"id":"mqbytlfk1u2","name":"GoldLoanRe-Payments","icon":"⚡","sectionType":"deduction","sheetName":"GoldLoanRe_Payments","columns":[{"key":"date","label":"Date","type":"date"},{"key":"name","label":"Name","type":"text"},{"key":"amount","label":"Amount","type":"number"},{"key":"notes","label":"Notes","type":"text"}]},{"id":"mqcd9ax3mcg","name":"Partial Outs","icon":"📁","sectionType":"investment","sheetName":"Partial_Outs","columns":[{"key":"date","label":"Date","type":"date"},{"key":"name","label":"Name","type":"text"},{"key":"amount","label":"Amount","type":"number"},{"key":"status","label":"Status","type":"status"},{"key":"notes","label":"Notes / Other Details","type":"text"}]}]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -602,36 +573,30 @@
       <c r="F1" t="str">
         <v>notes</v>
       </c>
-      <c r="G1" t="str">
-        <v>returns_rate</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mqbxfp9z8n9</v>
+        <v>mqawkf50bya</v>
       </c>
       <c r="B2" t="str">
-        <v>2025-11-22</v>
+        <v>2024-01-01</v>
       </c>
       <c r="C2" t="str">
-        <v>Golden Home Projects</v>
+        <v>Zaggle</v>
       </c>
       <c r="D2">
-        <v>3200000</v>
+        <v>120896</v>
       </c>
       <c r="E2" t="str">
         <v>Active</v>
       </c>
       <c r="F2" t="str">
         <v/>
-      </c>
-      <c r="G2">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -660,21 +625,21 @@
         <v>notes</v>
       </c>
       <c r="G1" t="str">
-        <v>returns</v>
+        <v>returns_rate</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mqbxqggnpkv</v>
+        <v>mqbxfp9z8n9</v>
       </c>
       <c r="B2" t="str">
-        <v>2025-12-01</v>
+        <v>2025-11-22</v>
       </c>
       <c r="C2" t="str">
-        <v>PF Till 2025</v>
+        <v>Golden Home Projects</v>
       </c>
       <c r="D2">
-        <v>380000</v>
+        <v>3200000</v>
       </c>
       <c r="E2" t="str">
         <v>Active</v>
@@ -682,8 +647,8 @@
       <c r="F2" t="str">
         <v/>
       </c>
-      <c r="G2">
-        <v>7</v>
+      <c r="G2" t="str">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -695,6 +660,63 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="G1" t="str">
+        <v>returns</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mqbxqggnpkv</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-12-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>PF Till 2025</v>
+      </c>
+      <c r="D2">
+        <v>380000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
@@ -738,7 +760,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F8"/>
   <sheetData>

</xml_diff>

<commit_message>
Finance update 2026-06-19 08:01
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -4539,7 +4539,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4621,9 +4621,29 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mqkn3egn324</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="C5" t="str">
+        <v xml:space="preserve">Claude subscription </v>
+      </c>
+      <c r="D5" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E5">
+        <v>2326</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-21 02:17
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2205,19 +2205,19 @@
         <v>7.65</v>
       </c>
       <c r="G26" t="str">
-        <v>Active</v>
+        <v>Broken</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>2026-06-21</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>2026-06-21</v>
       </c>
       <c r="K26">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v/>
       </c>
       <c r="P26" t="str">
-        <v/>
+        <v xml:space="preserve"> | Closed: Closed to give suresh anna</v>
       </c>
     </row>
     <row r="27">
@@ -4629,7 +4629,7 @@
         <v>2026-06-19</v>
       </c>
       <c r="C5" t="str">
-        <v xml:space="preserve">Claude subscription </v>
+        <v>Claude subscription</v>
       </c>
       <c r="D5" t="str">
         <v>Other</v>
@@ -4649,7 +4649,7 @@
         <v>2026-06-19</v>
       </c>
       <c r="C6" t="str">
-        <v xml:space="preserve">Monthly expenses </v>
+        <v>Monthly expenses</v>
       </c>
       <c r="D6" t="str">
         <v>Utilities</v>

</xml_diff>

<commit_message>
Finance update 2026-06-21 02:18
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2232,7 +2232,7 @@
         <v/>
       </c>
       <c r="P26" t="str">
-        <v xml:space="preserve"> | Closed: Closed to give suresh anna</v>
+        <v>| Closed: Closed to give suresh anna</v>
       </c>
     </row>
     <row r="27">
@@ -3676,7 +3676,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4252,9 +4252,35 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>mqn5r1s12jn</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Suresh Anna</v>
+      </c>
+      <c r="D15">
+        <v>200000</v>
+      </c>
+      <c r="E15">
+        <v>18</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-21 02:20
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -3676,7 +3676,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4252,35 +4252,9 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>mqn5r1s12jn</v>
-      </c>
-      <c r="B15" t="str">
-        <v>2026-06-20</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Suresh Anna</v>
-      </c>
-      <c r="D15">
-        <v>200000</v>
-      </c>
-      <c r="E15">
-        <v>18</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Active</v>
-      </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finance update 2026-06-21 02:21
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2205,7 +2205,7 @@
         <v>7.65</v>
       </c>
       <c r="G26" t="str">
-        <v>Broken</v>
+        <v>Active</v>
       </c>
       <c r="H26" t="str">
         <v>2026-06-21</v>
@@ -2232,7 +2232,7 @@
         <v/>
       </c>
       <c r="P26" t="str">
-        <v>| Closed: Closed to give suresh anna</v>
+        <v/>
       </c>
     </row>
     <row r="27">

</xml_diff>

<commit_message>
Finance update 2026-06-21 02:22
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -2205,13 +2205,13 @@
         <v>7.65</v>
       </c>
       <c r="G26" t="str">
-        <v>Active</v>
+        <v>Broken</v>
       </c>
       <c r="H26" t="str">
         <v>2026-06-21</v>
       </c>
       <c r="I26">
-        <v>200000</v>
+        <v>200001</v>
       </c>
       <c r="J26" t="str">
         <v>2026-06-21</v>
@@ -2220,7 +2220,7 @@
         <v>200000</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" t="str">
         <v/>

</xml_diff>